<commit_message>
ch31ms-9. MergeSortVisualizer 사용으로 원상복귀. Performance Excel File Update.
</commit_message>
<xml_diff>
--- a/week05_ch3/ch2_z_sort_performance.xlsx
+++ b/week05_ch3/ch2_z_sort_performance.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="15" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="16" uniqueCount="9">
   <si>
     <t>Count</t>
   </si>
@@ -50,6 +50,9 @@
   <si>
     <t>Merge</t>
   </si>
+  <si>
+    <t>Merge-Ins</t>
+  </si>
 </sst>
 </file>
 
@@ -58,7 +61,7 @@
   <numFmts count="1">
     <numFmt numFmtId="176" formatCode="0.000_ "/>
   </numFmts>
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -71,6 +74,15 @@
       <sz val="8"/>
       <name val="맑은 고딕"/>
       <family val="2"/>
+      <charset val="129"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="맑은 고딕"/>
+      <family val="3"/>
       <charset val="129"/>
       <scheme val="minor"/>
     </font>
@@ -97,11 +109,14 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="176" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="176" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
@@ -170,7 +185,6 @@
           </a:p>
         </c:rich>
       </c:tx>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -988,7 +1002,6 @@
     </c:plotArea>
     <c:legend>
       <c:legendPos val="b"/>
-      <c:layout/>
       <c:overlay val="0"/>
       <c:spPr>
         <a:noFill/>
@@ -2142,67 +2155,67 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>2E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.0000000000000001E-3</c:v>
+                  <c:v>5.0000000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>8.9999999999999993E-3</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.2999999999999999E-2</c:v>
-                </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6E-2</c:v>
+                  <c:v>1.2E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.02</c:v>
+                  <c:v>1.4999999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.4E-2</c:v>
+                  <c:v>1.9E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
+                  <c:v>2.1999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.5000000000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>2.5999999999999999E-2</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>3.1E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>3.5000000000000003E-2</c:v>
-                </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.3999999999999999E-2</c:v>
+                  <c:v>0.04</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>7.3999999999999996E-2</c:v>
+                  <c:v>5.7000000000000002E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.11600000000000001</c:v>
+                  <c:v>8.8999999999999996E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.159</c:v>
+                  <c:v>0.114</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.19600000000000001</c:v>
+                  <c:v>0.14899999999999999</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.442</c:v>
+                  <c:v>0.32900000000000001</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.89800000000000002</c:v>
+                  <c:v>0.69799999999999995</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.4390000000000001</c:v>
+                  <c:v>1.099</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.1110000000000002</c:v>
+                  <c:v>1.591</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.7170000000000001</c:v>
+                  <c:v>1.9690000000000001</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.6840000000000002</c:v>
+                  <c:v>4.0679999999999996</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>11.622999999999999</c:v>
@@ -2223,6 +2236,213 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-E17A-45B6-90D1-A5286279065C}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'O(nlogn)'!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Merge-Ins</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'O(nlogn)'!$A$2:$A$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9000</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>40000</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>100000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>200000</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>300000</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>400000</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1000000</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2000000</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3000000</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4000000</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'O(nlogn)'!$G$2:$G$27</c:f>
+              <c:numCache>
+                <c:formatCode>0.000_ </c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.9999999999999993E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.6E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.9E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.4E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.5999999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.1999999999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.107</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.13800000000000001</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.28799999999999998</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.0409999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.504</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.865</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.85</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-ED31-46C9-90BE-70FDF1507B2F}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -2241,7 +2461,7 @@
         <c:axId val="160975359"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="5000000"/>
+          <c:max val="1000000"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="b"/>
@@ -2304,6 +2524,7 @@
         <c:axId val="160969535"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:max val="10"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -3526,67 +3747,67 @@
                   <c:v>0</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>3.0000000000000001E-3</c:v>
+                  <c:v>2E-3</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>6.0000000000000001E-3</c:v>
+                  <c:v>5.0000000000000001E-3</c:v>
                 </c:pt>
                 <c:pt idx="3">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
                   <c:v>8.9999999999999993E-3</c:v>
                 </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.2999999999999999E-2</c:v>
-                </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.6E-2</c:v>
+                  <c:v>1.2E-2</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.02</c:v>
+                  <c:v>1.4999999999999999E-2</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>2.4E-2</c:v>
+                  <c:v>1.9E-2</c:v>
                 </c:pt>
                 <c:pt idx="8">
+                  <c:v>2.1999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.5000000000000001E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
                   <c:v>2.5999999999999999E-2</c:v>
                 </c:pt>
-                <c:pt idx="9">
-                  <c:v>3.1E-2</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>3.5000000000000003E-2</c:v>
-                </c:pt>
                 <c:pt idx="11">
-                  <c:v>5.3999999999999999E-2</c:v>
+                  <c:v>0.04</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>7.3999999999999996E-2</c:v>
+                  <c:v>5.7000000000000002E-2</c:v>
                 </c:pt>
                 <c:pt idx="13">
-                  <c:v>0.11600000000000001</c:v>
+                  <c:v>8.8999999999999996E-2</c:v>
                 </c:pt>
                 <c:pt idx="14">
-                  <c:v>0.159</c:v>
+                  <c:v>0.114</c:v>
                 </c:pt>
                 <c:pt idx="15">
-                  <c:v>0.19600000000000001</c:v>
+                  <c:v>0.14899999999999999</c:v>
                 </c:pt>
                 <c:pt idx="16">
-                  <c:v>0.442</c:v>
+                  <c:v>0.32900000000000001</c:v>
                 </c:pt>
                 <c:pt idx="17">
-                  <c:v>0.89800000000000002</c:v>
+                  <c:v>0.69799999999999995</c:v>
                 </c:pt>
                 <c:pt idx="18">
-                  <c:v>1.4390000000000001</c:v>
+                  <c:v>1.099</c:v>
                 </c:pt>
                 <c:pt idx="19">
-                  <c:v>2.1110000000000002</c:v>
+                  <c:v>1.591</c:v>
                 </c:pt>
                 <c:pt idx="20">
-                  <c:v>2.7170000000000001</c:v>
+                  <c:v>1.9690000000000001</c:v>
                 </c:pt>
                 <c:pt idx="21">
-                  <c:v>5.6840000000000002</c:v>
+                  <c:v>4.0679999999999996</c:v>
                 </c:pt>
                 <c:pt idx="22">
                   <c:v>11.622999999999999</c:v>
@@ -3607,6 +3828,213 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-565E-4B24-B735-62110011AA78}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>'O(nlogn)'!$G$1</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Merge-Ins</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent6"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent6"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>'O(nlogn)'!$A$2:$A$27</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>100</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1000</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>2000</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>3000</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>4000</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>5000</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>6000</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>7000</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>8000</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>9000</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>10000</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>15000</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>20000</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>30000</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>40000</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>50000</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>100000</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>200000</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>300000</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>400000</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>500000</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>1000000</c:v>
+                </c:pt>
+                <c:pt idx="22">
+                  <c:v>2000000</c:v>
+                </c:pt>
+                <c:pt idx="23">
+                  <c:v>3000000</c:v>
+                </c:pt>
+                <c:pt idx="24">
+                  <c:v>4000000</c:v>
+                </c:pt>
+                <c:pt idx="25">
+                  <c:v>5000000</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>'O(nlogn)'!$G$2:$G$27</c:f>
+              <c:numCache>
+                <c:formatCode>0.000_ </c:formatCode>
+                <c:ptCount val="26"/>
+                <c:pt idx="0">
+                  <c:v>0</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>2E-3</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>5.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>7.0000000000000001E-3</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>8.9999999999999993E-3</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.4E-2</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.6E-2</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.9E-2</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>2.1999999999999999E-2</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>2.4E-2</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>3.5999999999999997E-2</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>5.1999999999999998E-2</c:v>
+                </c:pt>
+                <c:pt idx="13">
+                  <c:v>0.08</c:v>
+                </c:pt>
+                <c:pt idx="14">
+                  <c:v>0.107</c:v>
+                </c:pt>
+                <c:pt idx="15">
+                  <c:v>0.13800000000000001</c:v>
+                </c:pt>
+                <c:pt idx="16">
+                  <c:v>0.28799999999999998</c:v>
+                </c:pt>
+                <c:pt idx="17">
+                  <c:v>0.68</c:v>
+                </c:pt>
+                <c:pt idx="18">
+                  <c:v>1.0409999999999999</c:v>
+                </c:pt>
+                <c:pt idx="19">
+                  <c:v>1.504</c:v>
+                </c:pt>
+                <c:pt idx="20">
+                  <c:v>1.865</c:v>
+                </c:pt>
+                <c:pt idx="21">
+                  <c:v>3.85</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="1"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-2258-4606-A8CE-72F1E5B05842}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -6530,13 +6958,13 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:F29"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr defaultRowHeight="17" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10.1640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -6555,8 +6983,11 @@
       <c r="F1" t="s">
         <v>7</v>
       </c>
+      <c r="G1" t="s">
+        <v>8</v>
+      </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2">
         <v>100</v>
       </c>
@@ -6575,8 +7006,11 @@
       <c r="F2" s="1">
         <v>0</v>
       </c>
+      <c r="G2" s="1">
+        <v>0</v>
+      </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3">
         <v>1000</v>
       </c>
@@ -6593,10 +7027,13 @@
         <v>3.0000000000000001E-3</v>
       </c>
       <c r="F3" s="1">
-        <v>3.0000000000000001E-3</v>
+        <v>2E-3</v>
+      </c>
+      <c r="G3" s="1">
+        <v>2E-3</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4">
         <v>2000</v>
       </c>
@@ -6613,10 +7050,13 @@
         <v>5.0000000000000001E-3</v>
       </c>
       <c r="F4" s="1">
-        <v>6.0000000000000001E-3</v>
+        <v>5.0000000000000001E-3</v>
+      </c>
+      <c r="G4" s="1">
+        <v>5.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5">
         <v>3000</v>
       </c>
@@ -6633,10 +7073,13 @@
         <v>8.9999999999999993E-3</v>
       </c>
       <c r="F5" s="1">
-        <v>8.9999999999999993E-3</v>
+        <v>7.0000000000000001E-3</v>
+      </c>
+      <c r="G5" s="1">
+        <v>7.0000000000000001E-3</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6">
         <v>4000</v>
       </c>
@@ -6653,10 +7096,13 @@
         <v>1.0999999999999999E-2</v>
       </c>
       <c r="F6" s="1">
-        <v>1.2999999999999999E-2</v>
+        <v>8.9999999999999993E-3</v>
+      </c>
+      <c r="G6" s="1">
+        <v>8.9999999999999993E-3</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7">
         <v>5000</v>
       </c>
@@ -6673,10 +7119,13 @@
         <v>1.2999999999999999E-2</v>
       </c>
       <c r="F7" s="1">
-        <v>1.6E-2</v>
+        <v>1.2E-2</v>
+      </c>
+      <c r="G7" s="1">
+        <v>1.0999999999999999E-2</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8">
         <v>6000</v>
       </c>
@@ -6693,10 +7142,13 @@
         <v>1.7999999999999999E-2</v>
       </c>
       <c r="F8" s="1">
-        <v>0.02</v>
+        <v>1.4999999999999999E-2</v>
+      </c>
+      <c r="G8" s="1">
+        <v>1.4E-2</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9">
         <v>7000</v>
       </c>
@@ -6713,10 +7165,13 @@
         <v>1.9E-2</v>
       </c>
       <c r="F9" s="1">
-        <v>2.4E-2</v>
+        <v>1.9E-2</v>
+      </c>
+      <c r="G9" s="1">
+        <v>1.6E-2</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10">
         <v>8000</v>
       </c>
@@ -6733,10 +7188,13 @@
         <v>2.1999999999999999E-2</v>
       </c>
       <c r="F10" s="1">
-        <v>2.5999999999999999E-2</v>
+        <v>2.1999999999999999E-2</v>
+      </c>
+      <c r="G10" s="1">
+        <v>1.9E-2</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11">
         <v>9000</v>
       </c>
@@ -6753,10 +7211,13 @@
         <v>2.4E-2</v>
       </c>
       <c r="F11" s="1">
-        <v>3.1E-2</v>
+        <v>2.5000000000000001E-2</v>
+      </c>
+      <c r="G11" s="1">
+        <v>2.1999999999999999E-2</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12">
         <v>10000</v>
       </c>
@@ -6773,10 +7234,13 @@
         <v>2.7E-2</v>
       </c>
       <c r="F12" s="1">
-        <v>3.5000000000000003E-2</v>
+        <v>2.5999999999999999E-2</v>
+      </c>
+      <c r="G12" s="1">
+        <v>2.4E-2</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13">
         <v>15000</v>
       </c>
@@ -6793,10 +7257,13 @@
         <v>3.9E-2</v>
       </c>
       <c r="F13" s="1">
-        <v>5.3999999999999999E-2</v>
+        <v>0.04</v>
+      </c>
+      <c r="G13" s="1">
+        <v>3.5999999999999997E-2</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14">
         <v>20000</v>
       </c>
@@ -6813,10 +7280,13 @@
         <v>5.2999999999999999E-2</v>
       </c>
       <c r="F14" s="1">
-        <v>7.3999999999999996E-2</v>
+        <v>5.7000000000000002E-2</v>
+      </c>
+      <c r="G14" s="1">
+        <v>5.1999999999999998E-2</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15">
         <v>30000</v>
       </c>
@@ -6833,10 +7303,13 @@
         <v>8.2000000000000003E-2</v>
       </c>
       <c r="F15" s="1">
-        <v>0.11600000000000001</v>
+        <v>8.8999999999999996E-2</v>
+      </c>
+      <c r="G15" s="1">
+        <v>0.08</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16">
         <v>40000</v>
       </c>
@@ -6853,10 +7326,13 @@
         <v>0.104</v>
       </c>
       <c r="F16" s="1">
-        <v>0.159</v>
+        <v>0.114</v>
+      </c>
+      <c r="G16" s="1">
+        <v>0.107</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17">
         <v>50000</v>
       </c>
@@ -6873,10 +7349,13 @@
         <v>0.13900000000000001</v>
       </c>
       <c r="F17" s="1">
-        <v>0.19600000000000001</v>
+        <v>0.14899999999999999</v>
+      </c>
+      <c r="G17" s="1">
+        <v>0.13800000000000001</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18">
         <v>100000</v>
       </c>
@@ -6893,10 +7372,13 @@
         <v>0.28100000000000003</v>
       </c>
       <c r="F18" s="1">
-        <v>0.442</v>
+        <v>0.32900000000000001</v>
+      </c>
+      <c r="G18" s="1">
+        <v>0.28799999999999998</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19">
         <v>200000</v>
       </c>
@@ -6913,10 +7395,13 @@
         <v>0.59399999999999997</v>
       </c>
       <c r="F19" s="1">
-        <v>0.89800000000000002</v>
+        <v>0.69799999999999995</v>
+      </c>
+      <c r="G19" s="1">
+        <v>0.68</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A20">
         <v>300000</v>
       </c>
@@ -6933,10 +7418,13 @@
         <v>0.95699999999999996</v>
       </c>
       <c r="F20" s="1">
-        <v>1.4390000000000001</v>
+        <v>1.099</v>
+      </c>
+      <c r="G20" s="1">
+        <v>1.0409999999999999</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A21">
         <v>400000</v>
       </c>
@@ -6953,10 +7441,13 @@
         <v>1.3660000000000001</v>
       </c>
       <c r="F21" s="1">
-        <v>2.1110000000000002</v>
+        <v>1.591</v>
+      </c>
+      <c r="G21" s="1">
+        <v>1.504</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A22">
         <v>500000</v>
       </c>
@@ -6973,10 +7464,13 @@
         <v>1.7</v>
       </c>
       <c r="F22" s="1">
-        <v>2.7170000000000001</v>
+        <v>1.9690000000000001</v>
+      </c>
+      <c r="G22" s="1">
+        <v>1.865</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A23">
         <v>1000000</v>
       </c>
@@ -6993,10 +7487,13 @@
         <v>3.17</v>
       </c>
       <c r="F23" s="1">
-        <v>5.6840000000000002</v>
+        <v>4.0679999999999996</v>
+      </c>
+      <c r="G23" s="1">
+        <v>3.85</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A24">
         <v>2000000</v>
       </c>
@@ -7012,11 +7509,12 @@
       <c r="E24" s="1">
         <v>7.6630000000000003</v>
       </c>
-      <c r="F24" s="1">
+      <c r="F24" s="2">
         <v>11.622999999999999</v>
       </c>
+      <c r="G24" s="1"/>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A25">
         <v>3000000</v>
       </c>
@@ -7032,11 +7530,12 @@
       <c r="E25" s="1">
         <v>11.76</v>
       </c>
-      <c r="F25" s="1">
+      <c r="F25" s="2">
         <v>18.082000000000001</v>
       </c>
+      <c r="G25" s="1"/>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A26">
         <v>4000000</v>
       </c>
@@ -7052,11 +7551,12 @@
       <c r="E26" s="1">
         <v>15.379</v>
       </c>
-      <c r="F26" s="1">
+      <c r="F26" s="2">
         <v>24.509</v>
       </c>
+      <c r="G26" s="1"/>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A27">
         <v>5000000</v>
       </c>
@@ -7072,11 +7572,12 @@
       <c r="E27" s="1">
         <v>18.72</v>
       </c>
-      <c r="F27" s="1">
+      <c r="F27" s="2">
         <v>31.692</v>
       </c>
+      <c r="G27" s="1"/>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A28">
         <v>10000000</v>
       </c>
@@ -7090,7 +7591,7 @@
       </c>
       <c r="F28" s="1"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A29">
         <v>100000000</v>
       </c>

</xml_diff>